<commit_message>
Add official sources for helplines and fraud steps
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/civic_platform_grounding_data.xlsx
+++ b/data/civic_platform_grounding_data.xlsx
@@ -35,7 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Scenarios" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources_Registry'!$A$3:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources_Registry'!$A$3:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Helplines'!$A$3:$G$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Schemes'!$A$3:$P$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Personas_Tests'!$A$3:$O$8</definedName>
@@ -3003,7 +3003,7 @@
       <c r="C6" s="21" t="n"/>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>REAL_SOURCED</t>
+          <t>UNVERIFIED_SOURCE_NEEDED</t>
         </is>
       </c>
     </row>
@@ -3018,10 +3018,14 @@
           <t>Keep ready: your name, mobile number, nearest police station, district, bank name, amount, account or UPI ID debited, transaction IDs, and a short description of what happened.</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n"/>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>REAL_SOURCED</t>
+          <t>REAL_SOURCED (core details only)</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="13" min="1" max="1"/>
@@ -5487,13 +5491,177 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="23.85" customHeight="1" s="14"/>
-    <row r="34" ht="15" customHeight="1" s="14"/>
-    <row r="35" ht="23.85" customHeight="1" s="14"/>
-    <row r="36" ht="23.85" customHeight="1" s="14"/>
+    <row r="33" ht="23.85" customHeight="1" s="14">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>S35</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>National helpline directory (112 integrated helpline, 102 National Ambulance Service)</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>National Portal of India (India.gov.in, NIC)</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>https://www.india.gov.in/directory/helpline</t>
+        </is>
+      </c>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr">
+        <is>
+          <t>Health; Disaster</t>
+        </is>
+      </c>
+      <c r="G33" s="21" t="inlineStr">
+        <is>
+          <t>REAL_SOURCED; page opened and read 2026-10-14</t>
+        </is>
+      </c>
+      <c r="H33" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="23.85" customHeight="1" s="14">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>Lok Sabha reply on ERSS (Dial 112), single pan-India emergency number</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>Ministry of Home Affairs via PIB</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleasePage.aspx?PRID=1594669</t>
+        </is>
+      </c>
+      <c r="E34" s="21" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="F34" s="21" t="inlineStr">
+        <is>
+          <t>Health; Disaster</t>
+        </is>
+      </c>
+      <c r="G34" s="21" t="inlineStr">
+        <is>
+          <t>REAL_SOURCED; page opened and read 2026-10-14</t>
+        </is>
+      </c>
+      <c r="H34" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="23.85" customHeight="1" s="14">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>Health transport: 108 (National Ambulance Service), Himachal Pradesh page</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>National Health Mission, Himachal Pradesh</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>https://nhm.hp.gov.in/health-transport</t>
+        </is>
+      </c>
+      <c r="E35" s="21" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="G35" s="21" t="inlineStr">
+        <is>
+          <t>REAL_SOURCED (state page); page opened and read 2026-10-14</t>
+        </is>
+      </c>
+      <c r="H35" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="23.85" customHeight="1" s="14">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>I4C FAQ: calling 1930 and details to give</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>Indian Cybercrime Coordination Centre, Ministry of Home Affairs</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>https://i4c.mha.gov.in/FAQ.aspx</t>
+        </is>
+      </c>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>Fraud</t>
+        </is>
+      </c>
+      <c r="F36" s="21" t="inlineStr">
+        <is>
+          <t>Fraud shield</t>
+        </is>
+      </c>
+      <c r="G36" s="21" t="inlineStr">
+        <is>
+          <t>REAL_SOURCED; page opened and read 2026-10-14</t>
+        </is>
+      </c>
+      <c r="H36" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+    </row>
     <row r="37" ht="23.85" customHeight="1" s="14"/>
   </sheetData>
-  <autoFilter ref="A3:H32"/>
+  <autoFilter ref="A3:H36"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -8057,7 +8225,11 @@
           <t>Health; Disaster</t>
         </is>
       </c>
-      <c r="F4" s="21" t="n"/>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>S35; S36</t>
+        </is>
+      </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
           <t>REAL_SOURCED</t>
@@ -8090,10 +8262,14 @@
           <t>Health; Disaster</t>
         </is>
       </c>
-      <c r="F5" s="21" t="n"/>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
       <c r="G5" s="21" t="inlineStr">
         <is>
-          <t>REAL_SOURCED</t>
+          <t>REAL_SOURCED (state page)</t>
         </is>
       </c>
     </row>
@@ -8123,10 +8299,14 @@
           <t>Health</t>
         </is>
       </c>
-      <c r="F6" s="21" t="n"/>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>S35</t>
+        </is>
+      </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>REAL_SOURCED</t>
+          <t>REAL_SOURCED (number only; 'free' not confirmed)</t>
         </is>
       </c>
     </row>

</xml_diff>